<commit_message>
adding jira automation tool
</commit_message>
<xml_diff>
--- a/jira-testcase-generator/template.xlsx
+++ b/jira-testcase-generator/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubham.singh\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubham.singh\Documents\Timken_Automation_POC\POC on AI on Testing\jira-testcase-generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2E1C01-B93E-42F1-9616-8D8258CDEA94}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC31A03D-185E-4A2B-B001-0D65B23CDFB9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7430" xr2:uid="{129235BF-B34C-44B1-8A73-067E6556FA97}"/>
   </bookViews>
@@ -141,7 +141,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -152,7 +152,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -599,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533422D3-27E8-4A48-8D86-152E65210DDB}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
@@ -646,118 +645,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>